<commit_message>
adress issue fix and some client side points
</commit_message>
<xml_diff>
--- a/outputs/test_grafton_output.xlsx
+++ b/outputs/test_grafton_output.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Consistency Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Takeoff" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Consistency Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Takeoff" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -547,7 +547,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -605,7 +605,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8">
@@ -616,7 +616,7 @@
       </c>
       <c r="B8" s="7" t="inlineStr">
         <is>
-          <t>71.3%</t>
+          <t>74.3%</t>
         </is>
       </c>
     </row>
@@ -669,82 +669,82 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>Dimension mismatch for 1118 (Bedroom 3): Plans 1100H×1800W vs NatHERS 1100H×1810W (Difference: 10mm).</t>
+          <t>Dimension mismatch for 1118 (BED 2): Plans 1100H×1800W vs NatHERS 1100H×1810W (Difference: 10mm).</t>
         </is>
       </c>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>1118</t>
+          <t>1006</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>Type Mismatch</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>Type mismatch for 1118 (Bedroom 3): Plans 'awning' vs NatHERS 'sliding'.</t>
+          <t>Dimension Mismatch</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Dimension mismatch for 1006 (BED 1): Plans 1000H×600W vs NatHERS 1800H×600W (Difference: 800mm).</t>
         </is>
       </c>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>1115</t>
-        </is>
-      </c>
-      <c r="B16" s="7" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
+          <t>1105</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Missing in Plans</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Type mismatch for 1115 (BATH): Plans 'awning' vs NatHERS 'sliding'.</t>
+          <t>1105 (Bedroom 1) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="20" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>1006</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Dimension Mismatch</t>
-        </is>
-      </c>
-      <c r="C17" s="10" t="inlineStr">
-        <is>
-          <t>Dimension mismatch for 1006 (ens): Plans 1000H×600W vs NatHERS 1800H×600W (Difference: 800mm).</t>
+          <t>1117</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Missing in Plans</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>1117 (Bedroom 1) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="20" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>1806</t>
-        </is>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
-        <is>
-          <t>Type Mismatch</t>
+          <t>1105</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Missing in Plans</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t>Type mismatch for 1806 (WIR): Plans 'awning' vs NatHERS 'fixed'.</t>
+          <t>1105 (Bedroom 1) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="20" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>1105</t>
+          <t>1818</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -754,14 +754,14 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>1105 (Bedroom 1) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
+          <t>1818 (Bedroom 2) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>1117</t>
+          <t>1124</t>
         </is>
       </c>
       <c r="B20" s="11" t="inlineStr">
@@ -770,57 +770,6 @@
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>1117 (Bedroom 1) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="20" customHeight="1">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>1105</t>
-        </is>
-      </c>
-      <c r="B21" s="11" t="inlineStr">
-        <is>
-          <t>Missing in Plans</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>1105 (Bedroom 1) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="6" t="inlineStr">
-        <is>
-          <t>1818</t>
-        </is>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>Missing in Plans</t>
-        </is>
-      </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>1818 (Bedroom 2) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="6" t="inlineStr">
-        <is>
-          <t>1124</t>
-        </is>
-      </c>
-      <c r="B23" s="11" t="inlineStr">
-        <is>
-          <t>Missing in Plans</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>1124 (Kitchen/Living) listed in NatHERS but not found on floor plans. Verify location on drawings.</t>
         </is>
@@ -978,7 +927,7 @@
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="17" t="inlineStr">
         <is>
-          <t>Kitchen/Living</t>
+          <t>BED 2</t>
         </is>
       </c>
       <c r="B4" s="18" t="inlineStr">
@@ -994,7 +943,7 @@
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
-          <t>awning</t>
+          <t>fixed</t>
         </is>
       </c>
       <c r="F4" s="18" t="inlineStr">
@@ -1004,14 +953,14 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>Aluminium A SG Clear</t>
+          <t>Aluminium B SG Clear</t>
         </is>
       </c>
       <c r="H4" s="18" t="n">
         <v>6.7</v>
       </c>
       <c r="I4" s="18" t="n">
-        <v>0.57</v>
+        <v>0.7</v>
       </c>
       <c r="J4" s="17" t="inlineStr">
         <is>
@@ -1030,7 +979,7 @@
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="17" t="inlineStr">
         <is>
-          <t>Bedroom 3</t>
+          <t>BED 2</t>
         </is>
       </c>
       <c r="B5" s="18" t="inlineStr">
@@ -1082,7 +1031,7 @@
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>BATH</t>
+          <t>BED 2</t>
         </is>
       </c>
       <c r="B6" s="18" t="inlineStr">
@@ -1134,7 +1083,7 @@
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="17" t="inlineStr">
         <is>
-          <t>ens</t>
+          <t>BED 1</t>
         </is>
       </c>
       <c r="B7" s="18" t="inlineStr">
@@ -1186,7 +1135,7 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="17" t="inlineStr">
         <is>
-          <t>Kitchen/Living</t>
+          <t>BED 1</t>
         </is>
       </c>
       <c r="B8" s="18" t="inlineStr">
@@ -1238,7 +1187,7 @@
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="17" t="inlineStr">
         <is>
-          <t>Kitchen/Living</t>
+          <t>E/S</t>
         </is>
       </c>
       <c r="B9" s="18" t="inlineStr">
@@ -1259,7 +1208,7 @@
       </c>
       <c r="F9" s="18" t="inlineStr">
         <is>
-          <t>W</t>
+          <t>E</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
@@ -1290,7 +1239,7 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>WIR</t>
+          <t>E/S</t>
         </is>
       </c>
       <c r="B10" s="18" t="inlineStr">
@@ -1306,24 +1255,24 @@
       </c>
       <c r="E10" s="17" t="inlineStr">
         <is>
-          <t>fixed</t>
+          <t>awning</t>
         </is>
       </c>
       <c r="F10" s="18" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>W</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>Aluminium B SG Clear</t>
+          <t>Aluminium A SG Clear</t>
         </is>
       </c>
       <c r="H10" s="18" t="n">
         <v>6.7</v>
       </c>
       <c r="I10" s="18" t="n">
-        <v>0.7</v>
+        <v>0.57</v>
       </c>
       <c r="J10" s="17" t="inlineStr">
         <is>

</xml_diff>